<commit_message>
feat(importfiles): Preserve and update actual domain import template filenames (Orta Avrupa importSalesV4, importroomingV4, MasterData_v2, UNO_Dynamic) in Publish/260829/importfiles
</commit_message>
<xml_diff>
--- a/Uno_API/Uno_API/wwwroot/templates/ExcelSample1_ExcursionSales_Import.xlsx
+++ b/Uno_API/Uno_API/wwwroot/templates/ExcelSample1_ExcursionSales_Import.xlsx
@@ -3,7 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="ExcursionSales" sheetId="1" r:id="rId1"/>
+    <sheet name="ExcusionSales" sheetId="1" r:id="rId1"/>
+    <sheet name="BaseServices" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -430,7 +431,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>BVP01092026</v>
+        <v>BVP05072026</v>
       </c>
       <c r="B2" t="str">
         <v>Prague Castle Guided Tour</v>
@@ -459,7 +460,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>BVP01092026</v>
+        <v>BVP05072026</v>
       </c>
       <c r="B3" t="str">
         <v>Budapest Danube Dinner Cruise</v>
@@ -491,4 +492,75 @@
     <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Tour Code</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Service Category</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Description</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Quantity</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Unit Price (€)</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Total Amount (€)</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>BVP05072026</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Guide</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Professional Licensed Guide (7 Days)</v>
+      </c>
+      <c r="D2">
+        <v>7</v>
+      </c>
+      <c r="E2">
+        <v>150</v>
+      </c>
+      <c r="F2">
+        <v>1050</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>BVP05072026</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Transport</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Luxury Bus Budapest-Vienna-Prague</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>3200</v>
+      </c>
+      <c r="F3">
+        <v>3200</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>